<commit_message>
feat(forward): atualiza resultados oficiais de 11/10/2026 com 11 Greens e 1 Red
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-10.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-10.xlsx
@@ -1998,15 +1998,19 @@
       <c r="K22" t="n">
         <v>1.4</v>
       </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>AO Home Win</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -2066,15 +2070,19 @@
       <c r="K23" t="n">
         <v>1.39</v>
       </c>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">

</xml_diff>